<commit_message>
update(SAV): update dataset with most recent submission
</commit_message>
<xml_diff>
--- a/data-raw/Wilcox - SAV Table for SOE Report - David Wilcox.xlsx
+++ b/data-raw/Wilcox - SAV Table for SOE Report - David Wilcox.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\Current Projects\Annual Mapping\SOE Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAA87BEF-6C35-4B9E-BE18-9FEE8D561B83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A290746-17B7-43D4-A9F8-C42727D92D90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{13C8E3A2-E6FB-475A-AAE8-164943661608}"/>
+    <workbookView xWindow="28680" yWindow="0" windowWidth="29040" windowHeight="15720" xr2:uid="{13C8E3A2-E6FB-475A-AAE8-164943661608}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1162,9 +1162,10 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="321">
     <cellStyle name="20% - Accent1 2" xfId="47" xr:uid="{0AFE57F7-0DD4-4FD8-AA50-8CDD2920CE29}"/>
@@ -1617,10 +1618,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$A$3:$A$40</c:f>
+              <c:f>Sheet1!$A$3:$A$42</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="38"/>
+                <c:ptCount val="40"/>
                 <c:pt idx="0">
                   <c:v>1984</c:v>
                 </c:pt>
@@ -1734,16 +1735,22 @@
                 </c:pt>
                 <c:pt idx="37">
                   <c:v>2022</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>2023</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$B$3:$B$40</c:f>
+              <c:f>Sheet1!$B$3:$B$42</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0_);_(* \(#,##0\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="38"/>
+                <c:ptCount val="40"/>
                 <c:pt idx="0">
                   <c:v>6911.1724799999993</c:v>
                 </c:pt>
@@ -1857,6 +1864,12 @@
                 </c:pt>
                 <c:pt idx="37">
                   <c:v>19411.28</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>19823.36</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>20217.59</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1908,10 +1921,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$A$3:$A$40</c:f>
+              <c:f>Sheet1!$A$3:$A$42</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="38"/>
+                <c:ptCount val="40"/>
                 <c:pt idx="0">
                   <c:v>1984</c:v>
                 </c:pt>
@@ -2025,16 +2038,22 @@
                 </c:pt>
                 <c:pt idx="37">
                   <c:v>2022</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>2023</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$C$3:$C$40</c:f>
+              <c:f>Sheet1!$C$3:$C$42</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0_);_(* \(#,##0\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="38"/>
+                <c:ptCount val="40"/>
                 <c:pt idx="0">
                   <c:v>653.259996</c:v>
                 </c:pt>
@@ -2148,6 +2167,12 @@
                 </c:pt>
                 <c:pt idx="37">
                   <c:v>7175.05</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>3421.56</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>4729.83</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2199,10 +2224,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$A$3:$A$40</c:f>
+              <c:f>Sheet1!$A$3:$A$42</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="38"/>
+                <c:ptCount val="40"/>
                 <c:pt idx="0">
                   <c:v>1984</c:v>
                 </c:pt>
@@ -2316,16 +2341,22 @@
                 </c:pt>
                 <c:pt idx="37">
                   <c:v>2022</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>2023</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$D$3:$D$40</c:f>
+              <c:f>Sheet1!$D$3:$D$42</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0_);_(* \(#,##0\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="38"/>
+                <c:ptCount val="40"/>
                 <c:pt idx="0">
                   <c:v>15635.934671999999</c:v>
                 </c:pt>
@@ -2439,6 +2470,12 @@
                 </c:pt>
                 <c:pt idx="37">
                   <c:v>31376.26</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>38370.6</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>33030.53</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2496,10 +2533,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$A$3:$A$40</c:f>
+              <c:f>Sheet1!$A$3:$A$42</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="38"/>
+                <c:ptCount val="40"/>
                 <c:pt idx="0">
                   <c:v>1984</c:v>
                 </c:pt>
@@ -2613,16 +2650,22 @@
                 </c:pt>
                 <c:pt idx="37">
                   <c:v>2022</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>2023</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$E$3:$E$40</c:f>
+              <c:f>Sheet1!$E$3:$E$42</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0_);_(* \(#,##0\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="38"/>
+                <c:ptCount val="40"/>
                 <c:pt idx="0">
                   <c:v>15027.278031</c:v>
                 </c:pt>
@@ -2736,6 +2779,12 @@
                 </c:pt>
                 <c:pt idx="37">
                   <c:v>19462.32</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>21803.43</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>24799.62</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2787,10 +2836,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$A$3:$A$40</c:f>
+              <c:f>Sheet1!$A$3:$A$42</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="38"/>
+                <c:ptCount val="40"/>
                 <c:pt idx="0">
                   <c:v>1984</c:v>
                 </c:pt>
@@ -2904,16 +2953,22 @@
                 </c:pt>
                 <c:pt idx="37">
                   <c:v>2022</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>2023</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$F$3:$F$40</c:f>
+              <c:f>Sheet1!$F$3:$F$42</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0_);_(* \(#,##0\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="38"/>
+                <c:ptCount val="40"/>
                 <c:pt idx="0">
                   <c:v>38227.645178999999</c:v>
                 </c:pt>
@@ -3027,6 +3082,12 @@
                 </c:pt>
                 <c:pt idx="37">
                   <c:v>77424.91</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>83418.95</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>82777.56</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3276,6 +3337,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -3283,7 +3345,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -3881,7 +3942,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="8677362" cy="6291743"/>
+    <xdr:ext cx="8670421" cy="6284720"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
@@ -4207,7 +4268,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FC34370-29BA-42C8-B125-C46ECD3E6C9B}">
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
@@ -5002,28 +5063,55 @@
       <c r="F40" s="1">
         <v>77424.91</v>
       </c>
-      <c r="H40" s="1"/>
-      <c r="J40" s="1"/>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>2023</v>
       </c>
       <c r="B41" s="1">
-        <v>19804.150000000001</v>
+        <v>19823.36</v>
       </c>
       <c r="C41" s="1">
-        <v>3428.71</v>
+        <v>3421.56</v>
       </c>
       <c r="D41" s="1">
-        <v>37960.67</v>
+        <v>38370.6</v>
       </c>
       <c r="E41" s="1">
-        <v>21743.31</v>
+        <v>21803.43</v>
       </c>
       <c r="F41" s="1">
-        <v>82936.84</v>
-      </c>
+        <v>83418.95</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>2024</v>
+      </c>
+      <c r="B42" s="1">
+        <v>20217.59</v>
+      </c>
+      <c r="C42" s="1">
+        <v>4729.83</v>
+      </c>
+      <c r="D42" s="1">
+        <v>33030.53</v>
+      </c>
+      <c r="E42" s="1">
+        <v>24799.62</v>
+      </c>
+      <c r="F42" s="1">
+        <v>82777.56</v>
+      </c>
+      <c r="H42" s="1"/>
+      <c r="J42" s="1"/>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A46" s="2"/>
+      <c r="B46" s="2"/>
+      <c r="C46" s="2"/>
+      <c r="D46" s="2"/>
+      <c r="E46" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>